<commit_message>
feat(farmacia): add Excel Bridge Office Script processor
</commit_message>
<xml_diff>
--- a/templates/PROMueve_FH_Caceres_Bridge_DEMO.xlsx
+++ b/templates/PROMueve_FH_Caceres_Bridge_DEMO.xlsx
@@ -315,6 +315,235 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblBridgeVisitLines" displayName="tblBridgeVisitLines" ref="A1:AT2" headerRowCount="1">
+  <autoFilter ref="A1:AT2"/>
+  <tableColumns count="46">
+    <tableColumn id="1" name="visit_id"/>
+    <tableColumn id="2" name="visit_type"/>
+    <tableColumn id="3" name="line_id"/>
+    <tableColumn id="4" name="treatment_id"/>
+    <tableColumn id="5" name="patient_id"/>
+    <tableColumn id="6" name="event_id"/>
+    <tableColumn id="7" name="source_event_id"/>
+    <tableColumn id="8" name="source_row_id"/>
+    <tableColumn id="9" name="line_role"/>
+    <tableColumn id="10" name="is_primary_line"/>
+    <tableColumn id="11" name="line_status_at_event"/>
+    <tableColumn id="12" name="active_at_event"/>
+    <tableColumn id="13" name="line_drug_name"/>
+    <tableColumn id="14" name="line_active_ingredient"/>
+    <tableColumn id="15" name="line_presentation"/>
+    <tableColumn id="16" name="line_dose_text"/>
+    <tableColumn id="17" name="line_route"/>
+    <tableColumn id="18" name="line_schedule_code"/>
+    <tableColumn id="19" name="line_schedule_label"/>
+    <tableColumn id="20" name="line_schedule_other_text"/>
+    <tableColumn id="21" name="line_selected_drug_id"/>
+    <tableColumn id="22" name="line_catalog_source"/>
+    <tableColumn id="23" name="line_national_code"/>
+    <tableColumn id="24" name="line_registration_number"/>
+    <tableColumn id="25" name="dispensation_status"/>
+    <tableColumn id="26" name="dispensation_observations"/>
+    <tableColumn id="27" name="specific_review_status"/>
+    <tableColumn id="28" name="specific_review_reason"/>
+    <tableColumn id="29" name="therapeutic_movement_type"/>
+    <tableColumn id="30" name="new_dose_text"/>
+    <tableColumn id="31" name="new_schedule_code"/>
+    <tableColumn id="32" name="new_schedule_label"/>
+    <tableColumn id="33" name="new_schedule_other_text"/>
+    <tableColumn id="34" name="new_route"/>
+    <tableColumn id="35" name="movement_reason"/>
+    <tableColumn id="36" name="movement_effective_date"/>
+    <tableColumn id="37" name="suspension_status"/>
+    <tableColumn id="38" name="suspension_reason"/>
+    <tableColumn id="39" name="suspension_effective_date"/>
+    <tableColumn id="40" name="line_observations"/>
+    <tableColumn id="41" name="adherence_collection_status"/>
+    <tableColumn id="42" name="adherence_instrument"/>
+    <tableColumn id="43" name="adherence_result"/>
+    <tableColumn id="44" name="adherence_answers_json"/>
+    <tableColumn id="45" name="source_table"/>
+    <tableColumn id="46" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblBridgeObservations" displayName="tblBridgeObservations" ref="A1:O2" headerRowCount="1">
+  <autoFilter ref="A1:O2"/>
+  <tableColumns count="15">
+    <tableColumn id="1" name="observation_key"/>
+    <tableColumn id="2" name="event_id"/>
+    <tableColumn id="3" name="source_event_id"/>
+    <tableColumn id="4" name="patient_id"/>
+    <tableColumn id="5" name="scope_type"/>
+    <tableColumn id="6" name="scope_ref"/>
+    <tableColumn id="7" name="source_field"/>
+    <tableColumn id="8" name="source_json_path"/>
+    <tableColumn id="9" name="explicit_scope"/>
+    <tableColumn id="10" name="explicit_reference_field"/>
+    <tableColumn id="11" name="explicit_reference"/>
+    <tableColumn id="12" name="content_json"/>
+    <tableColumn id="13" name="source_table"/>
+    <tableColumn id="14" name="source_row_id"/>
+    <tableColumn id="15" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblBridgeProms" displayName="tblBridgeProms" ref="A1:M2" headerRowCount="1">
+  <autoFilter ref="A1:M2"/>
+  <tableColumns count="13">
+    <tableColumn id="1" name="prom_key"/>
+    <tableColumn id="2" name="event_id"/>
+    <tableColumn id="3" name="source_event_id"/>
+    <tableColumn id="4" name="patient_id"/>
+    <tableColumn id="5" name="visit_id"/>
+    <tableColumn id="6" name="visit_type"/>
+    <tableColumn id="7" name="source_field"/>
+    <tableColumn id="8" name="source_json_path"/>
+    <tableColumn id="9" name="instrument_ref"/>
+    <tableColumn id="10" name="content_json"/>
+    <tableColumn id="11" name="source_table"/>
+    <tableColumn id="12" name="source_row_id"/>
+    <tableColumn id="13" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblBridgeAdverseEvents" displayName="tblBridgeAdverseEvents" ref="A1:N2" headerRowCount="1">
+  <autoFilter ref="A1:N2"/>
+  <tableColumns count="14">
+    <tableColumn id="1" name="adverse_event_id"/>
+    <tableColumn id="2" name="event_id"/>
+    <tableColumn id="3" name="source_event_id"/>
+    <tableColumn id="4" name="patient_id"/>
+    <tableColumn id="5" name="visit_id"/>
+    <tableColumn id="6" name="status"/>
+    <tableColumn id="7" name="description"/>
+    <tableColumn id="8" name="severity"/>
+    <tableColumn id="9" name="resolution_status"/>
+    <tableColumn id="10" name="action"/>
+    <tableColumn id="11" name="suspects_json"/>
+    <tableColumn id="12" name="source_table"/>
+    <tableColumn id="13" name="source_row_id"/>
+    <tableColumn id="14" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tblBridgeCausality" displayName="tblBridgeCausality" ref="A1:O2" headerRowCount="1">
+  <autoFilter ref="A1:O2"/>
+  <tableColumns count="15">
+    <tableColumn id="1" name="causality_key"/>
+    <tableColumn id="2" name="adverse_event_id"/>
+    <tableColumn id="3" name="event_id"/>
+    <tableColumn id="4" name="source_event_id"/>
+    <tableColumn id="5" name="patient_id"/>
+    <tableColumn id="6" name="visit_id"/>
+    <tableColumn id="7" name="suspect_ref"/>
+    <tableColumn id="8" name="method"/>
+    <tableColumn id="9" name="result"/>
+    <tableColumn id="10" name="score"/>
+    <tableColumn id="11" name="content_json"/>
+    <tableColumn id="12" name="source_json_path"/>
+    <tableColumn id="13" name="source_table"/>
+    <tableColumn id="14" name="source_row_id"/>
+    <tableColumn id="15" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblBridgeRenewalCycles" displayName="tblBridgeRenewalCycles" ref="A1:L2" headerRowCount="1">
+  <autoFilter ref="A1:L2"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="renewal_cycle_id"/>
+    <tableColumn id="2" name="line_id"/>
+    <tableColumn id="3" name="patient_id"/>
+    <tableColumn id="4" name="event_id"/>
+    <tableColumn id="5" name="source_event_id"/>
+    <tableColumn id="6" name="status"/>
+    <tableColumn id="7" name="confirmed_date"/>
+    <tableColumn id="8" name="verified_date"/>
+    <tableColumn id="9" name="estimated_date"/>
+    <tableColumn id="10" name="source_table"/>
+    <tableColumn id="11" name="source_row_id"/>
+    <tableColumn id="12" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tblBridgeRenewalTasks" displayName="tblBridgeRenewalTasks" ref="A1:K2" headerRowCount="1">
+  <autoFilter ref="A1:K2"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="renewal_task_id"/>
+    <tableColumn id="2" name="renewal_cycle_id"/>
+    <tableColumn id="3" name="line_id"/>
+    <tableColumn id="4" name="patient_id"/>
+    <tableColumn id="5" name="status"/>
+    <tableColumn id="6" name="due_at"/>
+    <tableColumn id="7" name="event_id"/>
+    <tableColumn id="8" name="source_event_id"/>
+    <tableColumn id="9" name="source_table"/>
+    <tableColumn id="10" name="source_row_id"/>
+    <tableColumn id="11" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tblBridgeAuditEvents" displayName="tblBridgeAuditEvents" ref="A1:L2" headerRowCount="1">
+  <autoFilter ref="A1:L2"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="audit_key"/>
+    <tableColumn id="2" name="processed_at"/>
+    <tableColumn id="3" name="outcome"/>
+    <tableColumn id="4" name="source_table"/>
+    <tableColumn id="5" name="source_physical_rows_json"/>
+    <tableColumn id="6" name="event_id"/>
+    <tableColumn id="7" name="source_event_id"/>
+    <tableColumn id="8" name="row_count"/>
+    <tableColumn id="9" name="row_ids_json"/>
+    <tableColumn id="10" name="entity_counts_json"/>
+    <tableColumn id="11" name="error_code"/>
+    <tableColumn id="12" name="error_detail"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tblBridgeImportErrors" displayName="tblBridgeImportErrors" ref="A1:J2" headerRowCount="1">
+  <autoFilter ref="A1:J2"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="error_key"/>
+    <tableColumn id="2" name="occurred_at"/>
+    <tableColumn id="3" name="source_table"/>
+    <tableColumn id="4" name="source_physical_row"/>
+    <tableColumn id="5" name="event_id"/>
+    <tableColumn id="6" name="source_event_id"/>
+    <tableColumn id="7" name="row_ids_json"/>
+    <tableColumn id="8" name="error_code"/>
+    <tableColumn id="9" name="error_detail"/>
+    <tableColumn id="10" name="raw_preserved"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblBridgeDigestivoInput" displayName="tblBridgeDigestivoInput" ref="A1:EV2" headerRowCount="1">
   <autoFilter ref="A1:EV2"/>
@@ -471,6 +700,234 @@
     <tableColumn id="150" name="adverse_event_action"/>
     <tableColumn id="151" name="adverse_event_suspects_json"/>
     <tableColumn id="152" name="causality_assessments_json"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblBridgePatients" displayName="tblBridgePatients" ref="A1:J2" headerRowCount="1">
+  <autoFilter ref="A1:J2"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="patient_id"/>
+    <tableColumn id="2" name="identifier_system"/>
+    <tableColumn id="3" name="identifier_value"/>
+    <tableColumn id="4" name="hospital_code"/>
+    <tableColumn id="5" name="demo_flag"/>
+    <tableColumn id="6" name="first_seen_event_id"/>
+    <tableColumn id="7" name="first_seen_source_event_id"/>
+    <tableColumn id="8" name="first_seen_source_table"/>
+    <tableColumn id="9" name="first_seen_source_row_id"/>
+    <tableColumn id="10" name="first_seen_processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblBridgeRequests" displayName="tblBridgeRequests" ref="A1:AI2" headerRowCount="1">
+  <autoFilter ref="A1:AI2"/>
+  <tableColumns count="35">
+    <tableColumn id="1" name="request_id"/>
+    <tableColumn id="2" name="patient_id"/>
+    <tableColumn id="3" name="event_id"/>
+    <tableColumn id="4" name="source_event_id"/>
+    <tableColumn id="5" name="event_status"/>
+    <tableColumn id="6" name="occurred_at"/>
+    <tableColumn id="7" name="recorded_at"/>
+    <tableColumn id="8" name="hospital_code"/>
+    <tableColumn id="9" name="service_code"/>
+    <tableColumn id="10" name="pathology_code"/>
+    <tableColumn id="11" name="professional_ref"/>
+    <tableColumn id="12" name="request_origin"/>
+    <tableColumn id="13" name="request_date"/>
+    <tableColumn id="14" name="validation_type"/>
+    <tableColumn id="15" name="pharmacy_appointment_date"/>
+    <tableColumn id="16" name="requested_drug_name"/>
+    <tableColumn id="17" name="requested_active_ingredient"/>
+    <tableColumn id="18" name="requested_presentation"/>
+    <tableColumn id="19" name="requested_dose_text"/>
+    <tableColumn id="20" name="requested_route"/>
+    <tableColumn id="21" name="requested_schedule_code"/>
+    <tableColumn id="22" name="requested_schedule_label"/>
+    <tableColumn id="23" name="requested_schedule_other_text"/>
+    <tableColumn id="24" name="requested_induction_status"/>
+    <tableColumn id="25" name="requested_weight_text"/>
+    <tableColumn id="26" name="requested_justification"/>
+    <tableColumn id="27" name="request_source_observations"/>
+    <tableColumn id="28" name="requested_selected_drug_id"/>
+    <tableColumn id="29" name="requested_catalog_source"/>
+    <tableColumn id="30" name="requested_national_code"/>
+    <tableColumn id="31" name="requested_registration_number"/>
+    <tableColumn id="32" name="demo_flag"/>
+    <tableColumn id="33" name="source_table"/>
+    <tableColumn id="34" name="source_row_id"/>
+    <tableColumn id="35" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblBridgeValidations" displayName="tblBridgeValidations" ref="A1:BC2" headerRowCount="1">
+  <autoFilter ref="A1:BC2"/>
+  <tableColumns count="55">
+    <tableColumn id="1" name="validation_id"/>
+    <tableColumn id="2" name="request_id"/>
+    <tableColumn id="3" name="patient_id"/>
+    <tableColumn id="4" name="event_id"/>
+    <tableColumn id="5" name="source_event_id"/>
+    <tableColumn id="6" name="event_status"/>
+    <tableColumn id="7" name="occurred_at"/>
+    <tableColumn id="8" name="recorded_at"/>
+    <tableColumn id="9" name="hospital_code"/>
+    <tableColumn id="10" name="service_code"/>
+    <tableColumn id="11" name="pathology_code"/>
+    <tableColumn id="12" name="professional_ref"/>
+    <tableColumn id="13" name="validation_result"/>
+    <tableColumn id="14" name="validation_pending_reason"/>
+    <tableColumn id="15" name="validation_denial_reason"/>
+    <tableColumn id="16" name="pharmacy_observations"/>
+    <tableColumn id="17" name="other_validation_observations"/>
+    <tableColumn id="18" name="validated_treatment_relation"/>
+    <tableColumn id="19" name="validated_drug_name"/>
+    <tableColumn id="20" name="validated_active_ingredient"/>
+    <tableColumn id="21" name="validated_presentation"/>
+    <tableColumn id="22" name="validated_dose_text"/>
+    <tableColumn id="23" name="validated_route"/>
+    <tableColumn id="24" name="validated_schedule_code"/>
+    <tableColumn id="25" name="validated_schedule_label"/>
+    <tableColumn id="26" name="validated_schedule_other_text"/>
+    <tableColumn id="27" name="validated_induction_status"/>
+    <tableColumn id="28" name="validated_selected_drug_id"/>
+    <tableColumn id="29" name="validated_catalog_source"/>
+    <tableColumn id="30" name="validated_national_code"/>
+    <tableColumn id="31" name="validated_registration_number"/>
+    <tableColumn id="32" name="validated_treatment_id"/>
+    <tableColumn id="33" name="validated_line_id"/>
+    <tableColumn id="34" name="line_creation_status"/>
+    <tableColumn id="35" name="prebiologic_required"/>
+    <tableColumn id="36" name="prebiologic_overall_status"/>
+    <tableColumn id="37" name="analysis_date"/>
+    <tableColumn id="38" name="analysis_recent_status"/>
+    <tableColumn id="39" name="hemogram_verified"/>
+    <tableColumn id="40" name="biochemistry_verified"/>
+    <tableColumn id="41" name="tb_status"/>
+    <tableColumn id="42" name="hbv_status"/>
+    <tableColumn id="43" name="hcv_status"/>
+    <tableColumn id="44" name="hiv_status"/>
+    <tableColumn id="45" name="vaccination_status"/>
+    <tableColumn id="46" name="vaccination_observations"/>
+    <tableColumn id="47" name="preventive_medicine_status"/>
+    <tableColumn id="48" name="recurrent_infections_status"/>
+    <tableColumn id="49" name="cardiovascular_risk_status"/>
+    <tableColumn id="50" name="neurologic_disorder_status"/>
+    <tableColumn id="51" name="neoplasia_history_or_risk_status"/>
+    <tableColumn id="52" name="demo_flag"/>
+    <tableColumn id="53" name="source_table"/>
+    <tableColumn id="54" name="source_row_id"/>
+    <tableColumn id="55" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblBridgeTreatments" displayName="tblBridgeTreatments" ref="A1:G2" headerRowCount="1">
+  <autoFilter ref="A1:G2"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="treatment_id"/>
+    <tableColumn id="2" name="patient_id"/>
+    <tableColumn id="3" name="first_seen_event_id"/>
+    <tableColumn id="4" name="first_seen_source_event_id"/>
+    <tableColumn id="5" name="first_seen_source_table"/>
+    <tableColumn id="6" name="first_seen_source_row_id"/>
+    <tableColumn id="7" name="first_seen_processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblBridgeTreatmentLines" displayName="tblBridgeTreatmentLines" ref="A1:H2" headerRowCount="1">
+  <autoFilter ref="A1:H2"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="line_id"/>
+    <tableColumn id="2" name="treatment_id"/>
+    <tableColumn id="3" name="patient_id"/>
+    <tableColumn id="4" name="first_seen_event_id"/>
+    <tableColumn id="5" name="first_seen_source_event_id"/>
+    <tableColumn id="6" name="first_seen_source_table"/>
+    <tableColumn id="7" name="first_seen_source_row_id"/>
+    <tableColumn id="8" name="first_seen_processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblBridgeTreatmentMovements" displayName="tblBridgeTreatmentMovements" ref="A1:T2" headerRowCount="1">
+  <autoFilter ref="A1:T2"/>
+  <tableColumns count="20">
+    <tableColumn id="1" name="movement_key"/>
+    <tableColumn id="2" name="event_id"/>
+    <tableColumn id="3" name="source_event_id"/>
+    <tableColumn id="4" name="source_row_id"/>
+    <tableColumn id="5" name="patient_id"/>
+    <tableColumn id="6" name="treatment_id"/>
+    <tableColumn id="7" name="line_id"/>
+    <tableColumn id="8" name="therapeutic_movement_type"/>
+    <tableColumn id="9" name="new_dose_text"/>
+    <tableColumn id="10" name="new_schedule_code"/>
+    <tableColumn id="11" name="new_schedule_label"/>
+    <tableColumn id="12" name="new_schedule_other_text"/>
+    <tableColumn id="13" name="new_route"/>
+    <tableColumn id="14" name="movement_reason"/>
+    <tableColumn id="15" name="movement_effective_date"/>
+    <tableColumn id="16" name="suspension_status"/>
+    <tableColumn id="17" name="suspension_reason"/>
+    <tableColumn id="18" name="suspension_effective_date"/>
+    <tableColumn id="19" name="source_table"/>
+    <tableColumn id="20" name="processed_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblBridgeVisits" displayName="tblBridgeVisits" ref="A1:AD2" headerRowCount="1">
+  <autoFilter ref="A1:AD2"/>
+  <tableColumns count="30">
+    <tableColumn id="1" name="visit_id"/>
+    <tableColumn id="2" name="visit_type"/>
+    <tableColumn id="3" name="patient_id"/>
+    <tableColumn id="4" name="event_id"/>
+    <tableColumn id="5" name="source_event_id"/>
+    <tableColumn id="6" name="event_status"/>
+    <tableColumn id="7" name="occurred_at"/>
+    <tableColumn id="8" name="recorded_at"/>
+    <tableColumn id="9" name="visit_date"/>
+    <tableColumn id="10" name="hospital_code"/>
+    <tableColumn id="11" name="service_code"/>
+    <tableColumn id="12" name="service_label"/>
+    <tableColumn id="13" name="pathology_code"/>
+    <tableColumn id="14" name="pathology_label"/>
+    <tableColumn id="15" name="professional_ref"/>
+    <tableColumn id="16" name="professional_display"/>
+    <tableColumn id="17" name="induction_performed_status"/>
+    <tableColumn id="18" name="stratification_level"/>
+    <tableColumn id="19" name="baseline_proms_collection_status"/>
+    <tableColumn id="20" name="pharmacy_visit_notes"/>
+    <tableColumn id="21" name="stratification_review_status"/>
+    <tableColumn id="22" name="previous_stratification_level"/>
+    <tableColumn id="23" name="new_stratification_level"/>
+    <tableColumn id="24" name="stratification_change_reason"/>
+    <tableColumn id="25" name="followup_proms_collection_status"/>
+    <tableColumn id="26" name="visit_general_observations"/>
+    <tableColumn id="27" name="demo_flag"/>
+    <tableColumn id="28" name="source_table"/>
+    <tableColumn id="29" name="source_row_id"/>
+    <tableColumn id="30" name="processed_at"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1852,10 +2309,342 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AT2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="14" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="17" customWidth="1" style="1" min="7" max="7"/>
+    <col width="15" customWidth="1" style="1" min="8" max="8"/>
+    <col width="12" customWidth="1" style="1" min="9" max="9"/>
+    <col width="17" customWidth="1" style="1" min="10" max="10"/>
+    <col width="22" customWidth="1" style="1" min="11" max="11"/>
+    <col width="17" customWidth="1" style="1" min="12" max="12"/>
+    <col width="16" customWidth="1" style="1" min="13" max="13"/>
+    <col width="24" customWidth="1" style="1" min="14" max="14"/>
+    <col width="19" customWidth="1" style="1" min="15" max="15"/>
+    <col width="16" customWidth="1" style="1" min="16" max="16"/>
+    <col width="12" customWidth="1" style="1" min="17" max="17"/>
+    <col width="20" customWidth="1" style="1" min="18" max="18"/>
+    <col width="21" customWidth="1" style="1" min="19" max="19"/>
+    <col width="26" customWidth="1" style="1" min="20" max="20"/>
+    <col width="23" customWidth="1" style="1" min="21" max="21"/>
+    <col width="21" customWidth="1" style="1" min="22" max="22"/>
+    <col width="20" customWidth="1" style="1" min="23" max="23"/>
+    <col width="26" customWidth="1" style="1" min="24" max="24"/>
+    <col width="21" customWidth="1" style="1" min="25" max="25"/>
+    <col width="27" customWidth="1" style="1" min="26" max="26"/>
+    <col width="24" customWidth="1" style="1" min="27" max="27"/>
+    <col width="24" customWidth="1" style="1" min="28" max="28"/>
+    <col width="27" customWidth="1" style="1" min="29" max="29"/>
+    <col width="15" customWidth="1" style="1" min="30" max="30"/>
+    <col width="19" customWidth="1" style="1" min="31" max="31"/>
+    <col width="20" customWidth="1" style="1" min="32" max="32"/>
+    <col width="25" customWidth="1" style="1" min="33" max="33"/>
+    <col width="12" customWidth="1" style="1" min="34" max="34"/>
+    <col width="17" customWidth="1" style="1" min="35" max="35"/>
+    <col width="25" customWidth="1" style="1" min="36" max="36"/>
+    <col width="19" customWidth="1" style="1" min="37" max="37"/>
+    <col width="19" customWidth="1" style="1" min="38" max="38"/>
+    <col width="27" customWidth="1" style="1" min="39" max="39"/>
+    <col width="19" customWidth="1" style="1" min="40" max="40"/>
+    <col width="28" customWidth="1" style="1" min="41" max="41"/>
+    <col width="22" customWidth="1" style="1" min="42" max="42"/>
+    <col width="18" customWidth="1" style="1" min="43" max="43"/>
+    <col width="24" customWidth="1" style="1" min="44" max="44"/>
+    <col width="14" customWidth="1" style="1" min="45" max="45"/>
+    <col width="14" customWidth="1" style="1" min="46" max="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>visit_type</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>line_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>treatment_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>line_role</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>is_primary_line</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>line_status_at_event</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>active_at_event</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>line_drug_name</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>line_active_ingredient</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>line_presentation</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>line_dose_text</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>line_route</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>line_schedule_code</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>line_schedule_label</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>line_schedule_other_text</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>line_selected_drug_id</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>line_catalog_source</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>line_national_code</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>line_registration_number</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>dispensation_status</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>dispensation_observations</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>specific_review_status</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>specific_review_reason</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>therapeutic_movement_type</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>new_dose_text</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>new_schedule_code</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>new_schedule_label</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>new_schedule_other_text</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>new_route</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>movement_reason</t>
+        </is>
+      </c>
+      <c r="AJ1" s="2" t="inlineStr">
+        <is>
+          <t>movement_effective_date</t>
+        </is>
+      </c>
+      <c r="AK1" s="2" t="inlineStr">
+        <is>
+          <t>suspension_status</t>
+        </is>
+      </c>
+      <c r="AL1" s="2" t="inlineStr">
+        <is>
+          <t>suspension_reason</t>
+        </is>
+      </c>
+      <c r="AM1" s="2" t="inlineStr">
+        <is>
+          <t>suspension_effective_date</t>
+        </is>
+      </c>
+      <c r="AN1" s="2" t="inlineStr">
+        <is>
+          <t>line_observations</t>
+        </is>
+      </c>
+      <c r="AO1" s="2" t="inlineStr">
+        <is>
+          <t>adherence_collection_status</t>
+        </is>
+      </c>
+      <c r="AP1" s="2" t="inlineStr">
+        <is>
+          <t>adherence_instrument</t>
+        </is>
+      </c>
+      <c r="AQ1" s="2" t="inlineStr">
+        <is>
+          <t>adherence_result</t>
+        </is>
+      </c>
+      <c r="AR1" s="2" t="inlineStr">
+        <is>
+          <t>adherence_answers_json</t>
+        </is>
+      </c>
+      <c r="AS1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="n"/>
+      <c r="W2" s="1" t="n"/>
+      <c r="X2" s="1" t="n"/>
+      <c r="Y2" s="1" t="n"/>
+      <c r="Z2" s="1" t="n"/>
+      <c r="AA2" s="1" t="n"/>
+      <c r="AB2" s="1" t="n"/>
+      <c r="AC2" s="1" t="n"/>
+      <c r="AD2" s="1" t="n"/>
+      <c r="AE2" s="1" t="n"/>
+      <c r="AF2" s="1" t="n"/>
+      <c r="AG2" s="1" t="n"/>
+      <c r="AH2" s="1" t="n"/>
+      <c r="AI2" s="1" t="n"/>
+      <c r="AJ2" s="1" t="n"/>
+      <c r="AK2" s="1" t="n"/>
+      <c r="AL2" s="1" t="n"/>
+      <c r="AM2" s="1" t="n"/>
+      <c r="AN2" s="1" t="n"/>
+      <c r="AO2" s="1" t="n"/>
+      <c r="AP2" s="1" t="n"/>
+      <c r="AQ2" s="1" t="n"/>
+      <c r="AR2" s="1" t="n"/>
+      <c r="AS2" s="1" t="n"/>
+      <c r="AT2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1865,10 +2654,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="17" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="17" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="14" customWidth="1" style="1" min="7" max="7"/>
+    <col width="18" customWidth="1" style="1" min="8" max="8"/>
+    <col width="16" customWidth="1" style="1" min="9" max="9"/>
+    <col width="26" customWidth="1" style="1" min="10" max="10"/>
+    <col width="20" customWidth="1" style="1" min="11" max="11"/>
+    <col width="14" customWidth="1" style="1" min="12" max="12"/>
+    <col width="14" customWidth="1" style="1" min="13" max="13"/>
+    <col width="15" customWidth="1" style="1" min="14" max="14"/>
+    <col width="14" customWidth="1" style="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>observation_key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>scope_type</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>scope_ref</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>source_field</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>source_json_path</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>explicit_scope</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>explicit_reference_field</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>explicit_reference</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>content_json</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1878,10 +2782,111 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="17" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="14" customWidth="1" style="1" min="7" max="7"/>
+    <col width="18" customWidth="1" style="1" min="8" max="8"/>
+    <col width="16" customWidth="1" style="1" min="9" max="9"/>
+    <col width="14" customWidth="1" style="1" min="10" max="10"/>
+    <col width="14" customWidth="1" style="1" min="11" max="11"/>
+    <col width="15" customWidth="1" style="1" min="12" max="12"/>
+    <col width="14" customWidth="1" style="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>prom_key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>visit_type</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>source_field</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>source_json_path</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>instrument_ref</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>content_json</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1891,10 +2896,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="17" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="13" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="1" min="8" max="8"/>
+    <col width="19" customWidth="1" style="1" min="9" max="9"/>
+    <col width="12" customWidth="1" style="1" min="10" max="10"/>
+    <col width="15" customWidth="1" style="1" min="11" max="11"/>
+    <col width="14" customWidth="1" style="1" min="12" max="12"/>
+    <col width="15" customWidth="1" style="1" min="13" max="13"/>
+    <col width="14" customWidth="1" style="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>adverse_event_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>resolution_status</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>suspects_json</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1904,10 +3017,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="15" customWidth="1" style="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="17" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="13" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="1" min="8" max="8"/>
+    <col width="12" customWidth="1" style="1" min="9" max="9"/>
+    <col width="12" customWidth="1" style="1" min="10" max="10"/>
+    <col width="14" customWidth="1" style="1" min="11" max="11"/>
+    <col width="18" customWidth="1" style="1" min="12" max="12"/>
+    <col width="14" customWidth="1" style="1" min="13" max="13"/>
+    <col width="15" customWidth="1" style="1" min="14" max="14"/>
+    <col width="14" customWidth="1" style="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>causality_key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>adverse_event_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>suspect_ref</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>content_json</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>source_json_path</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1917,10 +3145,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="1" min="4" max="4"/>
+    <col width="17" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="16" customWidth="1" style="1" min="7" max="7"/>
+    <col width="15" customWidth="1" style="1" min="8" max="8"/>
+    <col width="16" customWidth="1" style="1" min="9" max="9"/>
+    <col width="14" customWidth="1" style="1" min="10" max="10"/>
+    <col width="15" customWidth="1" style="1" min="11" max="11"/>
+    <col width="14" customWidth="1" style="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>renewal_cycle_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>line_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>confirmed_date</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>verified_date</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>estimated_date</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1930,10 +3252,97 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="17" customWidth="1" style="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="12" customWidth="1" style="1" min="7" max="7"/>
+    <col width="17" customWidth="1" style="1" min="8" max="8"/>
+    <col width="14" customWidth="1" style="1" min="9" max="9"/>
+    <col width="15" customWidth="1" style="1" min="10" max="10"/>
+    <col width="14" customWidth="1" style="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>renewal_task_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>renewal_cycle_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>line_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>due_at</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1943,10 +3352,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="14" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="14" customWidth="1" style="1" min="4" max="4"/>
+    <col width="27" customWidth="1" style="1" min="5" max="5"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="17" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="1" min="8" max="8"/>
+    <col width="14" customWidth="1" style="1" min="9" max="9"/>
+    <col width="20" customWidth="1" style="1" min="10" max="10"/>
+    <col width="12" customWidth="1" style="1" min="11" max="11"/>
+    <col width="14" customWidth="1" style="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>audit_key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>source_physical_rows_json</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>row_count</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>row_ids_json</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>entity_counts_json</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>error_code</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>error_detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1956,10 +3459,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="13" customWidth="1" style="1" min="2" max="2"/>
+    <col width="14" customWidth="1" style="1" min="3" max="3"/>
+    <col width="21" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="17" customWidth="1" style="1" min="6" max="6"/>
+    <col width="14" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="1" min="8" max="8"/>
+    <col width="14" customWidth="1" style="1" min="9" max="9"/>
+    <col width="15" customWidth="1" style="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>error_key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>occurred_at</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>source_physical_row</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>row_ids_json</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>error_code</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>error_detail</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>raw_preserved</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3056,10 +4639,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="19" customWidth="1" style="1" min="2" max="2"/>
+    <col width="18" customWidth="1" style="1" min="3" max="3"/>
+    <col width="15" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="21" customWidth="1" style="1" min="6" max="6"/>
+    <col width="28" customWidth="1" style="1" min="7" max="7"/>
+    <col width="25" customWidth="1" style="1" min="8" max="8"/>
+    <col width="26" customWidth="1" style="1" min="9" max="9"/>
+    <col width="25" customWidth="1" style="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>identifier_system</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>identifier_value</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>hospital_code</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>demo_flag</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_event_id</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_event_id</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_table</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_row_id</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3069,10 +4732,265 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="17" customWidth="1" style="1" min="4" max="4"/>
+    <col width="14" customWidth="1" style="1" min="5" max="5"/>
+    <col width="13" customWidth="1" style="1" min="6" max="6"/>
+    <col width="13" customWidth="1" style="1" min="7" max="7"/>
+    <col width="15" customWidth="1" style="1" min="8" max="8"/>
+    <col width="14" customWidth="1" style="1" min="9" max="9"/>
+    <col width="16" customWidth="1" style="1" min="10" max="10"/>
+    <col width="18" customWidth="1" style="1" min="11" max="11"/>
+    <col width="16" customWidth="1" style="1" min="12" max="12"/>
+    <col width="14" customWidth="1" style="1" min="13" max="13"/>
+    <col width="17" customWidth="1" style="1" min="14" max="14"/>
+    <col width="27" customWidth="1" style="1" min="15" max="15"/>
+    <col width="21" customWidth="1" style="1" min="16" max="16"/>
+    <col width="28" customWidth="1" style="1" min="17" max="17"/>
+    <col width="24" customWidth="1" style="1" min="18" max="18"/>
+    <col width="21" customWidth="1" style="1" min="19" max="19"/>
+    <col width="17" customWidth="1" style="1" min="20" max="20"/>
+    <col width="25" customWidth="1" style="1" min="21" max="21"/>
+    <col width="26" customWidth="1" style="1" min="22" max="22"/>
+    <col width="28" customWidth="1" style="1" min="23" max="23"/>
+    <col width="28" customWidth="1" style="1" min="24" max="24"/>
+    <col width="23" customWidth="1" style="1" min="25" max="25"/>
+    <col width="25" customWidth="1" style="1" min="26" max="26"/>
+    <col width="28" customWidth="1" style="1" min="27" max="27"/>
+    <col width="28" customWidth="1" style="1" min="28" max="28"/>
+    <col width="26" customWidth="1" style="1" min="29" max="29"/>
+    <col width="25" customWidth="1" style="1" min="30" max="30"/>
+    <col width="28" customWidth="1" style="1" min="31" max="31"/>
+    <col width="12" customWidth="1" style="1" min="32" max="32"/>
+    <col width="14" customWidth="1" style="1" min="33" max="33"/>
+    <col width="15" customWidth="1" style="1" min="34" max="34"/>
+    <col width="14" customWidth="1" style="1" min="35" max="35"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>request_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>event_status</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>occurred_at</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>recorded_at</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>hospital_code</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>service_code</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>pathology_code</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>professional_ref</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>request_origin</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>request_date</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>validation_type</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>pharmacy_appointment_date</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>requested_drug_name</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>requested_active_ingredient</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>requested_presentation</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>requested_dose_text</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>requested_route</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>requested_schedule_code</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>requested_schedule_label</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>requested_schedule_other_text</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>requested_induction_status</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>requested_weight_text</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>requested_justification</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>request_source_observations</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>requested_selected_drug_id</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>requested_catalog_source</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>requested_national_code</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>requested_registration_number</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>demo_flag</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="n"/>
+      <c r="W2" s="1" t="n"/>
+      <c r="X2" s="1" t="n"/>
+      <c r="Y2" s="1" t="n"/>
+      <c r="Z2" s="1" t="n"/>
+      <c r="AA2" s="1" t="n"/>
+      <c r="AB2" s="1" t="n"/>
+      <c r="AC2" s="1" t="n"/>
+      <c r="AD2" s="1" t="n"/>
+      <c r="AE2" s="1" t="n"/>
+      <c r="AF2" s="1" t="n"/>
+      <c r="AG2" s="1" t="n"/>
+      <c r="AH2" s="1" t="n"/>
+      <c r="AI2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3082,10 +5000,405 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:BC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="15" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="1" min="4" max="4"/>
+    <col width="17" customWidth="1" style="1" min="5" max="5"/>
+    <col width="14" customWidth="1" style="1" min="6" max="6"/>
+    <col width="13" customWidth="1" style="1" min="7" max="7"/>
+    <col width="13" customWidth="1" style="1" min="8" max="8"/>
+    <col width="15" customWidth="1" style="1" min="9" max="9"/>
+    <col width="14" customWidth="1" style="1" min="10" max="10"/>
+    <col width="16" customWidth="1" style="1" min="11" max="11"/>
+    <col width="18" customWidth="1" style="1" min="12" max="12"/>
+    <col width="19" customWidth="1" style="1" min="13" max="13"/>
+    <col width="27" customWidth="1" style="1" min="14" max="14"/>
+    <col width="26" customWidth="1" style="1" min="15" max="15"/>
+    <col width="23" customWidth="1" style="1" min="16" max="16"/>
+    <col width="28" customWidth="1" style="1" min="17" max="17"/>
+    <col width="28" customWidth="1" style="1" min="18" max="18"/>
+    <col width="21" customWidth="1" style="1" min="19" max="19"/>
+    <col width="28" customWidth="1" style="1" min="20" max="20"/>
+    <col width="24" customWidth="1" style="1" min="21" max="21"/>
+    <col width="21" customWidth="1" style="1" min="22" max="22"/>
+    <col width="17" customWidth="1" style="1" min="23" max="23"/>
+    <col width="25" customWidth="1" style="1" min="24" max="24"/>
+    <col width="26" customWidth="1" style="1" min="25" max="25"/>
+    <col width="28" customWidth="1" style="1" min="26" max="26"/>
+    <col width="28" customWidth="1" style="1" min="27" max="27"/>
+    <col width="28" customWidth="1" style="1" min="28" max="28"/>
+    <col width="26" customWidth="1" style="1" min="29" max="29"/>
+    <col width="25" customWidth="1" style="1" min="30" max="30"/>
+    <col width="28" customWidth="1" style="1" min="31" max="31"/>
+    <col width="24" customWidth="1" style="1" min="32" max="32"/>
+    <col width="19" customWidth="1" style="1" min="33" max="33"/>
+    <col width="22" customWidth="1" style="1" min="34" max="34"/>
+    <col width="22" customWidth="1" style="1" min="35" max="35"/>
+    <col width="28" customWidth="1" style="1" min="36" max="36"/>
+    <col width="15" customWidth="1" style="1" min="37" max="37"/>
+    <col width="24" customWidth="1" style="1" min="38" max="38"/>
+    <col width="19" customWidth="1" style="1" min="39" max="39"/>
+    <col width="23" customWidth="1" style="1" min="40" max="40"/>
+    <col width="12" customWidth="1" style="1" min="41" max="41"/>
+    <col width="12" customWidth="1" style="1" min="42" max="42"/>
+    <col width="12" customWidth="1" style="1" min="43" max="43"/>
+    <col width="12" customWidth="1" style="1" min="44" max="44"/>
+    <col width="20" customWidth="1" style="1" min="45" max="45"/>
+    <col width="26" customWidth="1" style="1" min="46" max="46"/>
+    <col width="28" customWidth="1" style="1" min="47" max="47"/>
+    <col width="28" customWidth="1" style="1" min="48" max="48"/>
+    <col width="28" customWidth="1" style="1" min="49" max="49"/>
+    <col width="28" customWidth="1" style="1" min="50" max="50"/>
+    <col width="28" customWidth="1" style="1" min="51" max="51"/>
+    <col width="12" customWidth="1" style="1" min="52" max="52"/>
+    <col width="14" customWidth="1" style="1" min="53" max="53"/>
+    <col width="15" customWidth="1" style="1" min="54" max="54"/>
+    <col width="14" customWidth="1" style="1" min="55" max="55"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>validation_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>request_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>event_status</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>occurred_at</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>recorded_at</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>hospital_code</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>service_code</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>pathology_code</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>professional_ref</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>validation_result</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>validation_pending_reason</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>validation_denial_reason</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>pharmacy_observations</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>other_validation_observations</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>validated_treatment_relation</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>validated_drug_name</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>validated_active_ingredient</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>validated_presentation</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>validated_dose_text</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>validated_route</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>validated_schedule_code</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>validated_schedule_label</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>validated_schedule_other_text</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>validated_induction_status</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>validated_selected_drug_id</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>validated_catalog_source</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>validated_national_code</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>validated_registration_number</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>validated_treatment_id</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>validated_line_id</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>line_creation_status</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>prebiologic_required</t>
+        </is>
+      </c>
+      <c r="AJ1" s="2" t="inlineStr">
+        <is>
+          <t>prebiologic_overall_status</t>
+        </is>
+      </c>
+      <c r="AK1" s="2" t="inlineStr">
+        <is>
+          <t>analysis_date</t>
+        </is>
+      </c>
+      <c r="AL1" s="2" t="inlineStr">
+        <is>
+          <t>analysis_recent_status</t>
+        </is>
+      </c>
+      <c r="AM1" s="2" t="inlineStr">
+        <is>
+          <t>hemogram_verified</t>
+        </is>
+      </c>
+      <c r="AN1" s="2" t="inlineStr">
+        <is>
+          <t>biochemistry_verified</t>
+        </is>
+      </c>
+      <c r="AO1" s="2" t="inlineStr">
+        <is>
+          <t>tb_status</t>
+        </is>
+      </c>
+      <c r="AP1" s="2" t="inlineStr">
+        <is>
+          <t>hbv_status</t>
+        </is>
+      </c>
+      <c r="AQ1" s="2" t="inlineStr">
+        <is>
+          <t>hcv_status</t>
+        </is>
+      </c>
+      <c r="AR1" s="2" t="inlineStr">
+        <is>
+          <t>hiv_status</t>
+        </is>
+      </c>
+      <c r="AS1" s="2" t="inlineStr">
+        <is>
+          <t>vaccination_status</t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
+        <is>
+          <t>vaccination_observations</t>
+        </is>
+      </c>
+      <c r="AU1" s="2" t="inlineStr">
+        <is>
+          <t>preventive_medicine_status</t>
+        </is>
+      </c>
+      <c r="AV1" s="2" t="inlineStr">
+        <is>
+          <t>recurrent_infections_status</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
+        <is>
+          <t>cardiovascular_risk_status</t>
+        </is>
+      </c>
+      <c r="AX1" s="2" t="inlineStr">
+        <is>
+          <t>neurologic_disorder_status</t>
+        </is>
+      </c>
+      <c r="AY1" s="2" t="inlineStr">
+        <is>
+          <t>neoplasia_history_or_risk_status</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
+        <is>
+          <t>demo_flag</t>
+        </is>
+      </c>
+      <c r="BA1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="BB1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="BC1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="n"/>
+      <c r="W2" s="1" t="n"/>
+      <c r="X2" s="1" t="n"/>
+      <c r="Y2" s="1" t="n"/>
+      <c r="Z2" s="1" t="n"/>
+      <c r="AA2" s="1" t="n"/>
+      <c r="AB2" s="1" t="n"/>
+      <c r="AC2" s="1" t="n"/>
+      <c r="AD2" s="1" t="n"/>
+      <c r="AE2" s="1" t="n"/>
+      <c r="AF2" s="1" t="n"/>
+      <c r="AG2" s="1" t="n"/>
+      <c r="AH2" s="1" t="n"/>
+      <c r="AI2" s="1" t="n"/>
+      <c r="AJ2" s="1" t="n"/>
+      <c r="AK2" s="1" t="n"/>
+      <c r="AL2" s="1" t="n"/>
+      <c r="AM2" s="1" t="n"/>
+      <c r="AN2" s="1" t="n"/>
+      <c r="AO2" s="1" t="n"/>
+      <c r="AP2" s="1" t="n"/>
+      <c r="AQ2" s="1" t="n"/>
+      <c r="AR2" s="1" t="n"/>
+      <c r="AS2" s="1" t="n"/>
+      <c r="AT2" s="1" t="n"/>
+      <c r="AU2" s="1" t="n"/>
+      <c r="AV2" s="1" t="n"/>
+      <c r="AW2" s="1" t="n"/>
+      <c r="AX2" s="1" t="n"/>
+      <c r="AY2" s="1" t="n"/>
+      <c r="AZ2" s="1" t="n"/>
+      <c r="BA2" s="1" t="n"/>
+      <c r="BB2" s="1" t="n"/>
+      <c r="BC2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3095,10 +5408,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="14" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="21" customWidth="1" style="1" min="3" max="3"/>
+    <col width="28" customWidth="1" style="1" min="4" max="4"/>
+    <col width="25" customWidth="1" style="1" min="5" max="5"/>
+    <col width="26" customWidth="1" style="1" min="6" max="6"/>
+    <col width="25" customWidth="1" style="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>treatment_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_event_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_event_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_table</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_row_id</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3108,10 +5480,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="14" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="21" customWidth="1" style="1" min="4" max="4"/>
+    <col width="28" customWidth="1" style="1" min="5" max="5"/>
+    <col width="25" customWidth="1" style="1" min="6" max="6"/>
+    <col width="26" customWidth="1" style="1" min="7" max="7"/>
+    <col width="25" customWidth="1" style="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>line_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>treatment_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_event_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_event_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_table</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_source_row_id</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>first_seen_processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3121,10 +5559,160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="14" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="17" customWidth="1" style="1" min="3" max="3"/>
+    <col width="15" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="14" customWidth="1" style="1" min="6" max="6"/>
+    <col width="12" customWidth="1" style="1" min="7" max="7"/>
+    <col width="27" customWidth="1" style="1" min="8" max="8"/>
+    <col width="15" customWidth="1" style="1" min="9" max="9"/>
+    <col width="19" customWidth="1" style="1" min="10" max="10"/>
+    <col width="20" customWidth="1" style="1" min="11" max="11"/>
+    <col width="25" customWidth="1" style="1" min="12" max="12"/>
+    <col width="12" customWidth="1" style="1" min="13" max="13"/>
+    <col width="17" customWidth="1" style="1" min="14" max="14"/>
+    <col width="25" customWidth="1" style="1" min="15" max="15"/>
+    <col width="19" customWidth="1" style="1" min="16" max="16"/>
+    <col width="19" customWidth="1" style="1" min="17" max="17"/>
+    <col width="27" customWidth="1" style="1" min="18" max="18"/>
+    <col width="14" customWidth="1" style="1" min="19" max="19"/>
+    <col width="14" customWidth="1" style="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>movement_key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>treatment_id</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>line_id</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>therapeutic_movement_type</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>new_dose_text</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>new_schedule_code</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>new_schedule_label</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>new_schedule_other_text</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>new_route</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>movement_reason</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>movement_effective_date</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>suspension_status</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>suspension_reason</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>suspension_effective_date</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3134,9 +5722,229 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AD2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12" customWidth="1" style="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="1" min="4" max="4"/>
+    <col width="17" customWidth="1" style="1" min="5" max="5"/>
+    <col width="14" customWidth="1" style="1" min="6" max="6"/>
+    <col width="13" customWidth="1" style="1" min="7" max="7"/>
+    <col width="13" customWidth="1" style="1" min="8" max="8"/>
+    <col width="12" customWidth="1" style="1" min="9" max="9"/>
+    <col width="15" customWidth="1" style="1" min="10" max="10"/>
+    <col width="14" customWidth="1" style="1" min="11" max="11"/>
+    <col width="15" customWidth="1" style="1" min="12" max="12"/>
+    <col width="16" customWidth="1" style="1" min="13" max="13"/>
+    <col width="17" customWidth="1" style="1" min="14" max="14"/>
+    <col width="18" customWidth="1" style="1" min="15" max="15"/>
+    <col width="22" customWidth="1" style="1" min="16" max="16"/>
+    <col width="28" customWidth="1" style="1" min="17" max="17"/>
+    <col width="22" customWidth="1" style="1" min="18" max="18"/>
+    <col width="28" customWidth="1" style="1" min="19" max="19"/>
+    <col width="22" customWidth="1" style="1" min="20" max="20"/>
+    <col width="28" customWidth="1" style="1" min="21" max="21"/>
+    <col width="28" customWidth="1" style="1" min="22" max="22"/>
+    <col width="26" customWidth="1" style="1" min="23" max="23"/>
+    <col width="28" customWidth="1" style="1" min="24" max="24"/>
+    <col width="28" customWidth="1" style="1" min="25" max="25"/>
+    <col width="28" customWidth="1" style="1" min="26" max="26"/>
+    <col width="12" customWidth="1" style="1" min="27" max="27"/>
+    <col width="14" customWidth="1" style="1" min="28" max="28"/>
+    <col width="15" customWidth="1" style="1" min="29" max="29"/>
+    <col width="14" customWidth="1" style="1" min="30" max="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>visit_type</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>patient_id</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>source_event_id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>event_status</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>occurred_at</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>recorded_at</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>visit_date</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>hospital_code</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>service_code</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>service_label</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>pathology_code</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>pathology_label</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>professional_ref</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>professional_display</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>induction_performed_status</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>stratification_level</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>baseline_proms_collection_status</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>pharmacy_visit_notes</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>stratification_review_status</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>previous_stratification_level</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>new_stratification_level</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>stratification_change_reason</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>followup_proms_collection_status</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>visit_general_observations</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>demo_flag</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>source_table</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>source_row_id</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>processed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="n"/>
+      <c r="W2" s="1" t="n"/>
+      <c r="X2" s="1" t="n"/>
+      <c r="Y2" s="1" t="n"/>
+      <c r="Z2" s="1" t="n"/>
+      <c r="AA2" s="1" t="n"/>
+      <c r="AB2" s="1" t="n"/>
+      <c r="AC2" s="1" t="n"/>
+      <c r="AD2" s="1" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>